<commit_message>
Change log, contratos multimoneda y documentación al día
- Change log: 6 entradas para las tarjetas del Resumen, la lectura del
  Contracts and Amendments, la etapa del proceso en el popup, la carga de
  archivos del portal y la actualización de README/manual.
- Contratos pagaderos en varias monedas (una fila por moneda en el
  Contracts and Amendments) muestran la suma de montos en vez de perder
  una de las filas (ej. CR-J0002-P00189).
- README y manual: operaciones que ya tienen Contracts and Amendments,
  contratos multimoneda y detalle por etapa en la tabla de tabs.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018djmuC1Qxi8SVjXpECHr3o
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -13963,7 +13963,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E112"/>
+  <dimension ref="A2:E118"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="3.7109375" customWidth="1" style="29" min="1" max="1"/>
@@ -16228,6 +16228,126 @@
         </is>
       </c>
     </row>
+    <row r="113">
+      <c r="B113" s="16" t="n">
+        <v>46302</v>
+      </c>
+      <c r="C113" s="15" t="inlineStr">
+        <is>
+          <t>Resumen</t>
+        </is>
+      </c>
+      <c r="D113" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E113" s="15" t="inlineStr">
+        <is>
+          <t>Tarjetas KPI del Resumen unificadas: Operaciones activas va primero; Cláusulas (vencidas / vencen ≤180 días), Productos críticos (retrasados / pausados) y Acuerdos (vencidos / vencen ≤30 días) muestran sus dos valores en una sola tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="16" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C114" s="15" t="inlineStr">
+        <is>
+          <t>Productos Críticos / Resultados</t>
+        </is>
+      </c>
+      <c r="D114" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E114" s="15" t="inlineStr">
+        <is>
+          <t>El popup de adquisición crítica muestra la etapa del proceso: si hay contrato, contratista, monto (moneda original), fecha de firma y fin estimado; si está previsto, fecha esperada de inicio; si está en curso, fecha esperada de firma del contrato</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="16" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C115" s="15" t="inlineStr">
+        <is>
+          <t>Raw Data</t>
+        </is>
+      </c>
+      <c r="D115" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E115" s="15" t="inlineStr">
+        <is>
+          <t>Se lee el nuevo archivo Contracts and Amendments (contratos registrados en el nuevo módulo del portal) junto con el Raw Data de cada operación; el archivo es opcional</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="B116" s="16" t="n">
+        <v>46303</v>
+      </c>
+      <c r="C116" s="15" t="inlineStr">
+        <is>
+          <t>Raw Data</t>
+        </is>
+      </c>
+      <c r="D116" s="15" t="inlineStr">
+        <is>
+          <t>CR-L1032, CR-L1139, CR-L1137, CR-J0002, CR-L1151, CR-L1157</t>
+        </is>
+      </c>
+      <c r="E116" s="15" t="inlineStr">
+        <is>
+          <t>Se actualizan los Raw Data de todas las operaciones y se agregan los Contracts and Amendments de 3071_OC-CR, 4864_OC-CR, 4871_OC-CR, 5777_GR-CR y 5823_OC-CR (6061_OC-CR no tiene)</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="B117" s="16" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C117" s="15" t="inlineStr">
+        <is>
+          <t>Productos Críticos / Resultados</t>
+        </is>
+      </c>
+      <c r="D117" s="15" t="inlineStr">
+        <is>
+          <t>CR-J0002</t>
+        </is>
+      </c>
+      <c r="E117" s="15" t="inlineStr">
+        <is>
+          <t>Los contratos pagaderos en varias monedas (una fila por moneda en Contracts and Amendments) muestran la suma de sus montos; p. ej. CR-J0002-P00189: CRC 1 610 690 000 + USD 550 500</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="B118" s="16" t="n">
+        <v>46304</v>
+      </c>
+      <c r="C118" s="15" t="inlineStr">
+        <is>
+          <t>README</t>
+        </is>
+      </c>
+      <c r="D118" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E118" s="15" t="inlineStr">
+        <is>
+          <t>Se actualizan README y manual Word: tarjetas del Resumen, archivo Contracts and Amendments, etapa del proceso en el popup de adquisición y operaciones que ya tienen el archivo complementario</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Raw Data y Contracts and Amendments desde la carpeta clientportal/
Los archivos del portal del cliente se movieron a clientportal/, así que
index.html dejaba de encontrarlos (404) y el popup de adquisiciones
críticas perdía nombre, estado, hitos y contratos. Se ajusta la ruta base.

README y manual Word: nueva ubicación de los archivos del portal y
descripción de las carpetas clientportal/ y pmr reports/ (esta última no
la lee el dashboard). Change log: una entrada nueva.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018djmuC1Qxi8SVjXpECHr3o
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -11971,7 +11971,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A2:E118"/>
+  <dimension ref="A2:E119"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -13620,6 +13620,26 @@
         <v>846</v>
       </c>
     </row>
+    <row r="119">
+      <c r="B119" s="16" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C119" s="15" t="inlineStr">
+        <is>
+          <t>Raw Data</t>
+        </is>
+      </c>
+      <c r="D119" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E119" s="15" t="inlineStr">
+        <is>
+          <t>Los Raw Data y Contracts and Amendments se movieron a la carpeta clientportal/; index.html ahora los busca ahí. README y manual Word actualizados con la nueva ubicación y la carpeta pmr reports/ (insumos del PMR, el dashboard no la lee)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Propuesta de visor Gantt de procesos de adquisición
Página nueva visor-adquisiciones.html (index.html no se modifica): una
barra por proceso con segmentos por fase de hitos del portal del cliente
(clientportal/ Raw Data + Contracts and Amendments), ejecución del
contrato, atrasos, filtros y detalle por proceso. Paleta de fases
validada para el fondo oscuro de la app; amarillo y rojo reservados para
estado como en index.html.

README, manual Word y change log actualizados.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018djmuC1Qxi8SVjXpECHr3o
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -11971,7 +11971,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A2:E119"/>
+  <dimension ref="A2:E120"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="3.7109375" customWidth="1"/>
@@ -13640,6 +13640,26 @@
         </is>
       </c>
     </row>
+    <row r="120">
+      <c r="B120" s="16" t="n">
+        <v>46311</v>
+      </c>
+      <c r="C120" s="15" t="inlineStr">
+        <is>
+          <t>Visor de adquisiciones</t>
+        </is>
+      </c>
+      <c r="D120" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E120" s="15" t="inlineStr">
+        <is>
+          <t>Propuesta de visor Gantt (visor-adquisiciones.html, página aparte de index.html): una barra por proceso segmentada por fase de hitos del portal del cliente, ejecución del contrato, atrasos y filtros; documentado en README y manual</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
update luego de skill de equipo de proyecto
</commit_message>
<xml_diff>
--- a/torre_de_control_CCR.xlsx
+++ b/torre_de_control_CCR.xlsx
@@ -14141,7 +14141,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:E124"/>
+  <dimension ref="A2:E125"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.109375" defaultRowHeight="14.4"/>
   <cols>
     <col width="3.6640625" customWidth="1" style="30" min="1" max="1"/>
@@ -16646,6 +16646,26 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="B125" s="16" t="n">
+        <v>46325</v>
+      </c>
+      <c r="C125" s="15" t="inlineStr">
+        <is>
+          <t>README</t>
+        </is>
+      </c>
+      <c r="D125" s="15" t="inlineStr">
+        <is>
+          <t>Todas</t>
+        </is>
+      </c>
+      <c r="E125" s="15" t="inlineStr">
+        <is>
+          <t>Se actualizan README y manual Word: nuevo skill torre-control-equipo-desde-convergencia (tabla de skills y sección "Barrido del equipo desde Convergencia"), regla de roles fijos en la hoja equipo y descripción de sus filas</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>